<commit_message>
Fix 26/10 no-overtime weekday ends 16:00 (not 15:30)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HsFNnGJRzg6EEfnut1VvMX
</commit_message>
<xml_diff>
--- a/loss-time/outputs/Danh_sach_sua_them_19-10_den_26-10.xlsx
+++ b/loss-time/outputs/Danh_sach_sua_them_19-10_den_26-10.xlsx
@@ -233,7 +233,7 @@
     <t xml:space="preserve">Chủ nhật 25/10 chỉ Assembly làm, không tăng ca</t>
   </si>
   <si>
-    <t xml:space="preserve">Thứ Hai 26/10 không tăng ca</t>
+    <t xml:space="preserve">Thứ Hai 26/10 không tăng ca (hết ca 16:00)</t>
   </si>
   <si>
     <t xml:space="preserve">Tổng</t>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C11" s="4" t="n">
         <f aca="false">SUMIFS('1. Nhập thêm'!$I$4:$I$99,'1. Nhập thêm'!$A$4:$A$99,A11)</f>
-        <v>339.5</v>
+        <v>349.5</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>0</v>
@@ -1293,10 +1293,10 @@
       </c>
       <c r="F11" s="4" t="n">
         <f aca="false">B11+C11+D11+E11</f>
-        <v>339.5</v>
+        <v>349.5</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>339.5</v>
+        <v>349.5</v>
       </c>
       <c r="H11" s="5" t="str">
         <f aca="false">IF(ABS(F11-G11)&lt;0.01,"Khớp","Lệch")</f>
@@ -3441,14 +3441,14 @@
         <v>0.3125</v>
       </c>
       <c r="G66" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H66" s="15" t="n">
         <v>2</v>
       </c>
       <c r="I66" s="12" t="n">
         <f aca="false">(G66-F66)*24*H66</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J66" s="13" t="s">
         <v>68</v>
@@ -3474,14 +3474,14 @@
         <v>0.3125</v>
       </c>
       <c r="G67" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H67" s="15" t="n">
         <v>4</v>
       </c>
       <c r="I67" s="12" t="n">
         <f aca="false">(G67-F67)*24*H67</f>
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J67" s="13" t="s">
         <v>68</v>
@@ -3507,14 +3507,14 @@
         <v>0.3125</v>
       </c>
       <c r="G68" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H68" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I68" s="12" t="n">
         <f aca="false">(G68-F68)*24*H68</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J68" s="13" t="s">
         <v>68</v>
@@ -3540,14 +3540,14 @@
         <v>0.3125</v>
       </c>
       <c r="G69" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H69" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I69" s="12" t="n">
         <f aca="false">(G69-F69)*24*H69</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J69" s="13" t="s">
         <v>68</v>
@@ -3573,14 +3573,14 @@
         <v>0.3125</v>
       </c>
       <c r="G70" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H70" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I70" s="12" t="n">
         <f aca="false">(G70-F70)*24*H70</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J70" s="13" t="s">
         <v>68</v>
@@ -3606,14 +3606,14 @@
         <v>0.3125</v>
       </c>
       <c r="G71" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H71" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I71" s="12" t="n">
         <f aca="false">(G71-F71)*24*H71</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J71" s="13" t="s">
         <v>68</v>
@@ -3639,14 +3639,14 @@
         <v>0.3125</v>
       </c>
       <c r="G72" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H72" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I72" s="12" t="n">
         <f aca="false">(G72-F72)*24*H72</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J72" s="13" t="s">
         <v>68</v>
@@ -3672,14 +3672,14 @@
         <v>0.3125</v>
       </c>
       <c r="G73" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H73" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I73" s="12" t="n">
         <f aca="false">(G73-F73)*24*H73</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J73" s="13" t="s">
         <v>68</v>
@@ -3705,14 +3705,14 @@
         <v>0.3125</v>
       </c>
       <c r="G74" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H74" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I74" s="12" t="n">
         <f aca="false">(G74-F74)*24*H74</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J74" s="13" t="s">
         <v>68</v>
@@ -3738,14 +3738,14 @@
         <v>0.3125</v>
       </c>
       <c r="G75" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H75" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I75" s="12" t="n">
         <f aca="false">(G75-F75)*24*H75</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J75" s="13" t="s">
         <v>68</v>
@@ -3771,14 +3771,14 @@
         <v>0.3125</v>
       </c>
       <c r="G76" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H76" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I76" s="12" t="n">
         <f aca="false">(G76-F76)*24*H76</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J76" s="13" t="s">
         <v>68</v>
@@ -3804,14 +3804,14 @@
         <v>0.3125</v>
       </c>
       <c r="G77" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H77" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I77" s="12" t="n">
         <f aca="false">(G77-F77)*24*H77</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J77" s="13" t="s">
         <v>68</v>
@@ -3837,14 +3837,14 @@
         <v>0.3125</v>
       </c>
       <c r="G78" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H78" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I78" s="12" t="n">
         <f aca="false">(G78-F78)*24*H78</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J78" s="13" t="s">
         <v>68</v>
@@ -3870,14 +3870,14 @@
         <v>0.3125</v>
       </c>
       <c r="G79" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H79" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I79" s="12" t="n">
         <f aca="false">(G79-F79)*24*H79</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J79" s="13" t="s">
         <v>68</v>
@@ -3903,14 +3903,14 @@
         <v>0.3125</v>
       </c>
       <c r="G80" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H80" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I80" s="12" t="n">
         <f aca="false">(G80-F80)*24*H80</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J80" s="13" t="s">
         <v>68</v>
@@ -3936,14 +3936,14 @@
         <v>0.3125</v>
       </c>
       <c r="G81" s="17" t="n">
-        <v>0.645833333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="H81" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I81" s="12" t="n">
         <f aca="false">(G81-F81)*24*H81</f>
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="J81" s="13" t="s">
         <v>68</v>
@@ -4549,7 +4549,7 @@
       </c>
       <c r="I100" s="19" t="n">
         <f aca="false">SUM(I4:I99)</f>
-        <v>879.5</v>
+        <v>889.5</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
26/10: weekday always overtime (restore standard P20/P26)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HsFNnGJRzg6EEfnut1VvMX
</commit_message>
<xml_diff>
--- a/loss-time/outputs/Danh_sach_sua_them_19-10_den_26-10.xlsx
+++ b/loss-time/outputs/Danh_sach_sua_them_19-10_den_26-10.xlsx
@@ -233,7 +233,7 @@
     <t xml:space="preserve">Chủ nhật 25/10 chỉ Assembly làm, không tăng ca</t>
   </si>
   <si>
-    <t xml:space="preserve">Thứ Hai 26/10 không tăng ca (hết ca 16:00)</t>
+    <t xml:space="preserve">Thứ Hai 26/10 (ngày thường, có tăng ca)</t>
   </si>
   <si>
     <t xml:space="preserve">Tổng</t>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C11" s="4" t="n">
         <f aca="false">SUMIFS('1. Nhập thêm'!$I$4:$I$99,'1. Nhập thêm'!$A$4:$A$99,A11)</f>
-        <v>349.5</v>
+        <v>429.5</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>0</v>
@@ -1293,10 +1293,10 @@
       </c>
       <c r="F11" s="4" t="n">
         <f aca="false">B11+C11+D11+E11</f>
-        <v>349.5</v>
+        <v>429.5</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>349.5</v>
+        <v>429.5</v>
       </c>
       <c r="H11" s="5" t="str">
         <f aca="false">IF(ABS(F11-G11)&lt;0.01,"Khớp","Lệch")</f>
@@ -3441,14 +3441,14 @@
         <v>0.3125</v>
       </c>
       <c r="G66" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H66" s="15" t="n">
         <v>2</v>
       </c>
       <c r="I66" s="12" t="n">
         <f aca="false">(G66-F66)*24*H66</f>
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="J66" s="13" t="s">
         <v>68</v>
@@ -3474,14 +3474,14 @@
         <v>0.3125</v>
       </c>
       <c r="G67" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H67" s="15" t="n">
         <v>4</v>
       </c>
       <c r="I67" s="12" t="n">
         <f aca="false">(G67-F67)*24*H67</f>
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="J67" s="13" t="s">
         <v>68</v>
@@ -3507,14 +3507,14 @@
         <v>0.3125</v>
       </c>
       <c r="G68" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H68" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I68" s="12" t="n">
         <f aca="false">(G68-F68)*24*H68</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J68" s="13" t="s">
         <v>68</v>
@@ -3540,14 +3540,14 @@
         <v>0.3125</v>
       </c>
       <c r="G69" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H69" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I69" s="12" t="n">
         <f aca="false">(G69-F69)*24*H69</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J69" s="13" t="s">
         <v>68</v>
@@ -3573,14 +3573,14 @@
         <v>0.3125</v>
       </c>
       <c r="G70" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H70" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I70" s="12" t="n">
         <f aca="false">(G70-F70)*24*H70</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J70" s="13" t="s">
         <v>68</v>
@@ -3606,14 +3606,14 @@
         <v>0.3125</v>
       </c>
       <c r="G71" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H71" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I71" s="12" t="n">
         <f aca="false">(G71-F71)*24*H71</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J71" s="13" t="s">
         <v>68</v>
@@ -3639,14 +3639,14 @@
         <v>0.3125</v>
       </c>
       <c r="G72" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H72" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I72" s="12" t="n">
         <f aca="false">(G72-F72)*24*H72</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J72" s="13" t="s">
         <v>68</v>
@@ -3672,14 +3672,14 @@
         <v>0.3125</v>
       </c>
       <c r="G73" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H73" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I73" s="12" t="n">
         <f aca="false">(G73-F73)*24*H73</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J73" s="13" t="s">
         <v>68</v>
@@ -3705,14 +3705,14 @@
         <v>0.3125</v>
       </c>
       <c r="G74" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H74" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I74" s="12" t="n">
         <f aca="false">(G74-F74)*24*H74</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J74" s="13" t="s">
         <v>68</v>
@@ -3738,14 +3738,14 @@
         <v>0.3125</v>
       </c>
       <c r="G75" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H75" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I75" s="12" t="n">
         <f aca="false">(G75-F75)*24*H75</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J75" s="13" t="s">
         <v>68</v>
@@ -3771,14 +3771,14 @@
         <v>0.3125</v>
       </c>
       <c r="G76" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H76" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I76" s="12" t="n">
         <f aca="false">(G76-F76)*24*H76</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J76" s="13" t="s">
         <v>68</v>
@@ -3804,14 +3804,14 @@
         <v>0.3125</v>
       </c>
       <c r="G77" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H77" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I77" s="12" t="n">
         <f aca="false">(G77-F77)*24*H77</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J77" s="13" t="s">
         <v>68</v>
@@ -3837,14 +3837,14 @@
         <v>0.3125</v>
       </c>
       <c r="G78" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H78" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I78" s="12" t="n">
         <f aca="false">(G78-F78)*24*H78</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J78" s="13" t="s">
         <v>68</v>
@@ -3870,14 +3870,14 @@
         <v>0.3125</v>
       </c>
       <c r="G79" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H79" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I79" s="12" t="n">
         <f aca="false">(G79-F79)*24*H79</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J79" s="13" t="s">
         <v>68</v>
@@ -3903,14 +3903,14 @@
         <v>0.3125</v>
       </c>
       <c r="G80" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H80" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I80" s="12" t="n">
         <f aca="false">(G80-F80)*24*H80</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J80" s="13" t="s">
         <v>68</v>
@@ -3936,14 +3936,14 @@
         <v>0.3125</v>
       </c>
       <c r="G81" s="17" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="H81" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I81" s="12" t="n">
         <f aca="false">(G81-F81)*24*H81</f>
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="J81" s="13" t="s">
         <v>68</v>
@@ -4549,7 +4549,7 @@
       </c>
       <c r="I100" s="19" t="n">
         <f aca="false">SUM(I4:I99)</f>
-        <v>889.5</v>
+        <v>969.5</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>